<commit_message>
Add round from 4/4/2026
</commit_message>
<xml_diff>
--- a/data/GolfData.xlsx
+++ b/data/GolfData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Apps\GolfStats\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F34FA9-3E88-41BB-B1CB-8A558CBB7931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DB6386-D1EE-42EA-A240-AEE20D8368B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29790" yWindow="4020" windowWidth="21600" windowHeight="11295" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Score Cards" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>Cypress Point</t>
+  </si>
+  <si>
+    <t>Sewells Point</t>
   </si>
 </sst>
 </file>
@@ -207,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -227,6 +230,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1184,8 +1190,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W18" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
-  <autoFilter ref="A1:W18" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W19" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+  <autoFilter ref="A1:W19" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
   <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{6036417A-52C2-4AF8-9A0D-25AEE607F48A}" name="Course" dataDxfId="70"/>
     <tableColumn id="2" xr3:uid="{AE08F17B-78CF-43B6-86B1-7635DA793064}" name="Date" dataDxfId="69"/>
@@ -1216,8 +1222,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BA24C5C8-325A-47BE-A13D-D90937A1910E}" name="Table2" displayName="Table2" ref="A1:S3" totalsRowShown="0" headerRowDxfId="47" dataDxfId="45" headerRowBorderDxfId="46" tableBorderDxfId="44">
-  <autoFilter ref="A1:S3" xr:uid="{BA24C5C8-325A-47BE-A13D-D90937A1910E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BA24C5C8-325A-47BE-A13D-D90937A1910E}" name="Table2" displayName="Table2" ref="A1:S4" totalsRowShown="0" headerRowDxfId="47" dataDxfId="45" headerRowBorderDxfId="46" tableBorderDxfId="44">
+  <autoFilter ref="A1:S4" xr:uid="{BA24C5C8-325A-47BE-A13D-D90937A1910E}"/>
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{DD6BC8FF-48C3-4E6B-8977-DC0A4AF98ADF}" name="Course" dataDxfId="43"/>
     <tableColumn id="2" xr3:uid="{DAD1FCCF-276C-4332-967F-D073C1E0DDD1}" name="1" dataDxfId="42"/>
@@ -1244,8 +1250,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E23CC1EA-99BC-4242-AF8E-4EFD850D2CFF}" name="Table24" displayName="Table24" ref="A1:U4" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21">
-  <autoFilter ref="A1:U4" xr:uid="{E23CC1EA-99BC-4242-AF8E-4EFD850D2CFF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E23CC1EA-99BC-4242-AF8E-4EFD850D2CFF}" name="Table24" displayName="Table24" ref="A1:U5" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21">
+  <autoFilter ref="A1:U5" xr:uid="{E23CC1EA-99BC-4242-AF8E-4EFD850D2CFF}"/>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{CFEBEA66-C11E-40EA-9B1C-519F8D6D5A4D}" name="Course" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{E3A55B99-6240-4A04-9BEC-04FB4FD27D1A}" name="1" dataDxfId="19"/>
@@ -1570,7 +1576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838B056B-02E7-4106-A28B-369A087ADF9A}">
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="1" customWidth="1"/>
@@ -2859,6 +2865,77 @@
         <v>5</v>
       </c>
     </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="2">
+        <v>46116</v>
+      </c>
+      <c r="C19" s="1">
+        <v>5</v>
+      </c>
+      <c r="D19" s="1">
+        <v>5</v>
+      </c>
+      <c r="E19" s="1">
+        <v>5</v>
+      </c>
+      <c r="F19" s="1">
+        <v>5</v>
+      </c>
+      <c r="G19" s="1">
+        <v>5</v>
+      </c>
+      <c r="H19" s="1">
+        <v>5</v>
+      </c>
+      <c r="I19" s="1">
+        <v>3</v>
+      </c>
+      <c r="J19" s="1">
+        <v>7</v>
+      </c>
+      <c r="K19" s="1">
+        <v>4</v>
+      </c>
+      <c r="L19" s="1">
+        <v>4</v>
+      </c>
+      <c r="M19" s="1">
+        <v>7</v>
+      </c>
+      <c r="N19" s="1">
+        <v>6</v>
+      </c>
+      <c r="O19" s="1">
+        <v>5</v>
+      </c>
+      <c r="P19" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>6</v>
+      </c>
+      <c r="R19" s="1">
+        <v>4</v>
+      </c>
+      <c r="S19" s="1">
+        <v>6</v>
+      </c>
+      <c r="T19" s="1">
+        <v>4</v>
+      </c>
+      <c r="U19" s="1">
+        <v>3</v>
+      </c>
+      <c r="V19" s="1">
+        <v>37</v>
+      </c>
+      <c r="W19" s="1">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2869,7 +2946,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A42EF0A-8226-4283-852A-2A86FD4BC582}">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -3050,6 +3127,65 @@
       </c>
       <c r="S3" s="1">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="7">
+        <v>9</v>
+      </c>
+      <c r="C4" s="7">
+        <v>13</v>
+      </c>
+      <c r="D4" s="7">
+        <v>7</v>
+      </c>
+      <c r="E4" s="7">
+        <v>17</v>
+      </c>
+      <c r="F4" s="7">
+        <v>3</v>
+      </c>
+      <c r="G4" s="7">
+        <v>5</v>
+      </c>
+      <c r="H4" s="7">
+        <v>15</v>
+      </c>
+      <c r="I4" s="7">
+        <v>11</v>
+      </c>
+      <c r="J4" s="7">
+        <v>1</v>
+      </c>
+      <c r="K4" s="7">
+        <v>16</v>
+      </c>
+      <c r="L4" s="7">
+        <v>6</v>
+      </c>
+      <c r="M4" s="7">
+        <v>10</v>
+      </c>
+      <c r="N4" s="7">
+        <v>4</v>
+      </c>
+      <c r="O4" s="7">
+        <v>12</v>
+      </c>
+      <c r="P4" s="7">
+        <v>8</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>18</v>
+      </c>
+      <c r="R4" s="7">
+        <v>2</v>
+      </c>
+      <c r="S4" s="7">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -3062,7 +3198,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{534A788D-C5D7-487E-983A-A68219D7D8C3}">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
@@ -3328,6 +3464,71 @@
         <v>118</v>
       </c>
     </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="7">
+        <v>4</v>
+      </c>
+      <c r="C5" s="7">
+        <v>4</v>
+      </c>
+      <c r="D5" s="7">
+        <v>4</v>
+      </c>
+      <c r="E5" s="7">
+        <v>3</v>
+      </c>
+      <c r="F5" s="7">
+        <v>4</v>
+      </c>
+      <c r="G5" s="7">
+        <v>5</v>
+      </c>
+      <c r="H5" s="7">
+        <v>3</v>
+      </c>
+      <c r="I5" s="7">
+        <v>4</v>
+      </c>
+      <c r="J5" s="7">
+        <v>4</v>
+      </c>
+      <c r="K5" s="7">
+        <v>3</v>
+      </c>
+      <c r="L5" s="7">
+        <v>5</v>
+      </c>
+      <c r="M5" s="7">
+        <v>4</v>
+      </c>
+      <c r="N5" s="7">
+        <v>4</v>
+      </c>
+      <c r="O5" s="7">
+        <v>4</v>
+      </c>
+      <c r="P5" s="7">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="7">
+        <v>3</v>
+      </c>
+      <c r="R5" s="7">
+        <v>4</v>
+      </c>
+      <c r="S5" s="7">
+        <v>4</v>
+      </c>
+      <c r="T5" s="7">
+        <v>68.2</v>
+      </c>
+      <c r="U5" s="7">
+        <v>121</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
add score from 27 JUN 2026
</commit_message>
<xml_diff>
--- a/data/GolfData.xlsx
+++ b/data/GolfData.xlsx
@@ -1,42 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Apps\GolfStats\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78DB6386-D1EE-42EA-A240-AEE20D8368B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01380EE7-31E4-4A60-A3A4-A5267B854F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4BA5778-8140-4272-B97C-07E35F2520D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Score Cards" sheetId="1" r:id="rId1"/>
     <sheet name="Course Handicaps" sheetId="2" r:id="rId2"/>
     <sheet name="Course Pars" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -210,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -230,9 +221,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1190,8 +1178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W19" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
-  <autoFilter ref="A1:W19" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}" name="Table1" displayName="Table1" ref="A1:W20" totalsRowShown="0" headerRowDxfId="74" dataDxfId="72" headerRowBorderDxfId="73" tableBorderDxfId="71">
+  <autoFilter ref="A1:W20" xr:uid="{67CDCE95-7C63-4EE1-A07D-718040E657E9}"/>
   <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{6036417A-52C2-4AF8-9A0D-25AEE607F48A}" name="Course" dataDxfId="70"/>
     <tableColumn id="2" xr3:uid="{AE08F17B-78CF-43B6-86B1-7635DA793064}" name="Date" dataDxfId="69"/>
@@ -1576,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838B056B-02E7-4106-A28B-369A087ADF9A}">
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="1" customWidth="1"/>
@@ -2933,6 +2921,77 @@
         <v>37</v>
       </c>
       <c r="W19" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2">
+        <v>46200</v>
+      </c>
+      <c r="C20" s="1">
+        <v>3</v>
+      </c>
+      <c r="D20" s="1">
+        <v>6</v>
+      </c>
+      <c r="E20" s="1">
+        <v>8</v>
+      </c>
+      <c r="F20" s="1">
+        <v>3</v>
+      </c>
+      <c r="G20" s="1">
+        <v>4</v>
+      </c>
+      <c r="H20" s="1">
+        <v>3</v>
+      </c>
+      <c r="I20" s="1">
+        <v>5</v>
+      </c>
+      <c r="J20" s="1">
+        <v>5</v>
+      </c>
+      <c r="K20" s="1">
+        <v>5</v>
+      </c>
+      <c r="L20" s="1">
+        <v>5</v>
+      </c>
+      <c r="M20" s="1">
+        <v>5</v>
+      </c>
+      <c r="N20" s="1">
+        <v>5</v>
+      </c>
+      <c r="O20" s="1">
+        <v>4</v>
+      </c>
+      <c r="P20" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q20" s="1">
+        <v>3</v>
+      </c>
+      <c r="R20" s="1">
+        <v>7</v>
+      </c>
+      <c r="S20" s="1">
+        <v>4</v>
+      </c>
+      <c r="T20" s="1">
+        <v>5</v>
+      </c>
+      <c r="U20" s="1">
+        <v>2</v>
+      </c>
+      <c r="V20" s="1">
+        <v>28</v>
+      </c>
+      <c r="W20" s="1">
         <v>7</v>
       </c>
     </row>
@@ -3133,58 +3192,58 @@
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="1">
         <v>9</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="1">
         <v>13</v>
       </c>
-      <c r="D4" s="7">
-        <v>7</v>
-      </c>
-      <c r="E4" s="7">
+      <c r="D4" s="1">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1">
         <v>17</v>
       </c>
-      <c r="F4" s="7">
-        <v>3</v>
-      </c>
-      <c r="G4" s="7">
-        <v>5</v>
-      </c>
-      <c r="H4" s="7">
+      <c r="F4" s="1">
+        <v>3</v>
+      </c>
+      <c r="G4" s="1">
+        <v>5</v>
+      </c>
+      <c r="H4" s="1">
         <v>15</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="1">
         <v>11</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="1">
         <v>1</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="1">
         <v>16</v>
       </c>
-      <c r="L4" s="7">
-        <v>6</v>
-      </c>
-      <c r="M4" s="7">
+      <c r="L4" s="1">
+        <v>6</v>
+      </c>
+      <c r="M4" s="1">
         <v>10</v>
       </c>
-      <c r="N4" s="7">
-        <v>4</v>
-      </c>
-      <c r="O4" s="7">
+      <c r="N4" s="1">
+        <v>4</v>
+      </c>
+      <c r="O4" s="1">
         <v>12</v>
       </c>
-      <c r="P4" s="7">
+      <c r="P4" s="1">
         <v>8</v>
       </c>
-      <c r="Q4" s="7">
+      <c r="Q4" s="1">
         <v>18</v>
       </c>
-      <c r="R4" s="7">
+      <c r="R4" s="1">
         <v>2</v>
       </c>
-      <c r="S4" s="7">
+      <c r="S4" s="1">
         <v>14</v>
       </c>
     </row>
@@ -3468,64 +3527,64 @@
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="7">
-        <v>4</v>
-      </c>
-      <c r="C5" s="7">
-        <v>4</v>
-      </c>
-      <c r="D5" s="7">
-        <v>4</v>
-      </c>
-      <c r="E5" s="7">
-        <v>3</v>
-      </c>
-      <c r="F5" s="7">
-        <v>4</v>
-      </c>
-      <c r="G5" s="7">
-        <v>5</v>
-      </c>
-      <c r="H5" s="7">
-        <v>3</v>
-      </c>
-      <c r="I5" s="7">
-        <v>4</v>
-      </c>
-      <c r="J5" s="7">
-        <v>4</v>
-      </c>
-      <c r="K5" s="7">
-        <v>3</v>
-      </c>
-      <c r="L5" s="7">
-        <v>5</v>
-      </c>
-      <c r="M5" s="7">
-        <v>4</v>
-      </c>
-      <c r="N5" s="7">
-        <v>4</v>
-      </c>
-      <c r="O5" s="7">
-        <v>4</v>
-      </c>
-      <c r="P5" s="7">
-        <v>5</v>
-      </c>
-      <c r="Q5" s="7">
-        <v>3</v>
-      </c>
-      <c r="R5" s="7">
-        <v>4</v>
-      </c>
-      <c r="S5" s="7">
-        <v>4</v>
-      </c>
-      <c r="T5" s="7">
+      <c r="B5" s="1">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1">
+        <v>4</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>4</v>
+      </c>
+      <c r="G5" s="1">
+        <v>5</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1">
+        <v>4</v>
+      </c>
+      <c r="J5" s="1">
+        <v>4</v>
+      </c>
+      <c r="K5" s="1">
+        <v>3</v>
+      </c>
+      <c r="L5" s="1">
+        <v>5</v>
+      </c>
+      <c r="M5" s="1">
+        <v>4</v>
+      </c>
+      <c r="N5" s="1">
+        <v>4</v>
+      </c>
+      <c r="O5" s="1">
+        <v>4</v>
+      </c>
+      <c r="P5" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>3</v>
+      </c>
+      <c r="R5" s="1">
+        <v>4</v>
+      </c>
+      <c r="S5" s="1">
+        <v>4</v>
+      </c>
+      <c r="T5" s="1">
         <v>68.2</v>
       </c>
-      <c r="U5" s="7">
+      <c r="U5" s="1">
         <v>121</v>
       </c>
     </row>

</xml_diff>